<commit_message>
Update ZONE buildings data
</commit_message>
<xml_diff>
--- a/data_xlsx/zone_struktura_budynkow_zrodla_co_polska.xlsx
+++ b/data_xlsx/zone_struktura_budynkow_zrodla_co_polska.xlsx
@@ -255,7 +255,7 @@
       <c r="C3" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">3 570 356</t>
+            <t xml:space="preserve">3 569 992</t>
           </r>
         </is>
       </c>
@@ -263,7 +263,7 @@
       <c r="E3" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">56.77</t>
+            <t xml:space="preserve">56.74</t>
           </r>
         </is>
       </c>
@@ -281,7 +281,7 @@
       <c r="C4" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">460 339</t>
+            <t xml:space="preserve">461 060</t>
           </r>
         </is>
       </c>
@@ -289,7 +289,7 @@
       <c r="E4" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">7.32</t>
+            <t xml:space="preserve">7.33</t>
           </r>
         </is>
       </c>
@@ -307,7 +307,7 @@
       <c r="C5" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">143 620</t>
+            <t xml:space="preserve">143 780</t>
           </r>
         </is>
       </c>
@@ -315,7 +315,7 @@
       <c r="E5" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">2.28</t>
+            <t xml:space="preserve">2.29</t>
           </r>
         </is>
       </c>
@@ -333,7 +333,7 @@
       <c r="C6" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">779 282</t>
+            <t xml:space="preserve">778 818</t>
           </r>
         </is>
       </c>
@@ -341,7 +341,7 @@
       <c r="E6" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">12.39</t>
+            <t xml:space="preserve">12.38</t>
           </r>
         </is>
       </c>
@@ -359,7 +359,7 @@
       <c r="C7" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">1 135 230</t>
+            <t xml:space="preserve">1 134 438</t>
           </r>
         </is>
       </c>
@@ -367,7 +367,7 @@
       <c r="E7" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">18.05</t>
+            <t xml:space="preserve">18.03</t>
           </r>
         </is>
       </c>
@@ -385,7 +385,7 @@
       <c r="C8" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">545 368</t>
+            <t xml:space="preserve">545 448</t>
           </r>
         </is>
       </c>
@@ -411,7 +411,7 @@
       <c r="C9" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">309 838</t>
+            <t xml:space="preserve">309 650</t>
           </r>
         </is>
       </c>
@@ -419,7 +419,7 @@
       <c r="E9" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">4.93</t>
+            <t xml:space="preserve">4.92</t>
           </r>
         </is>
       </c>
@@ -437,7 +437,7 @@
       <c r="C10" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">84 376</t>
+            <t xml:space="preserve">84 561</t>
           </r>
         </is>
       </c>
@@ -463,7 +463,7 @@
       <c r="C11" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">112 303</t>
+            <t xml:space="preserve">112 237</t>
           </r>
         </is>
       </c>
@@ -471,7 +471,7 @@
       <c r="E11" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">1.79</t>
+            <t xml:space="preserve">1.78</t>
           </r>
         </is>
       </c>
@@ -489,7 +489,7 @@
       <c r="C12" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">1 578 117</t>
+            <t xml:space="preserve">1 579 554</t>
           </r>
         </is>
       </c>
@@ -497,7 +497,7 @@
       <c r="E12" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">25.09</t>
+            <t xml:space="preserve">25.11</t>
           </r>
         </is>
       </c>
@@ -515,7 +515,7 @@
       <c r="C13" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">1 201 357</t>
+            <t xml:space="preserve">1 202 195</t>
           </r>
         </is>
       </c>
@@ -523,7 +523,7 @@
       <c r="E13" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">19.10</t>
+            <t xml:space="preserve">19.11</t>
           </r>
         </is>
       </c>
@@ -541,7 +541,7 @@
       <c r="C14" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">218 274</t>
+            <t xml:space="preserve">218 736</t>
           </r>
         </is>
       </c>
@@ -549,7 +549,7 @@
       <c r="E14" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">3.47</t>
+            <t xml:space="preserve">3.48</t>
           </r>
         </is>
       </c>
@@ -567,7 +567,7 @@
       <c r="C15" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">57 826</t>
+            <t xml:space="preserve">57 906</t>
           </r>
         </is>
       </c>
@@ -593,7 +593,7 @@
       <c r="C16" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">32 672</t>
+            <t xml:space="preserve">32 655</t>
           </r>
         </is>
       </c>
@@ -619,7 +619,7 @@
       <c r="C17" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">40 032</t>
+            <t xml:space="preserve">40 051</t>
           </r>
         </is>
       </c>
@@ -645,7 +645,7 @@
       <c r="C18" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">981</t>
+            <t xml:space="preserve">982</t>
           </r>
         </is>
       </c>
@@ -671,7 +671,7 @@
       <c r="C19" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">2 419</t>
+            <t xml:space="preserve">2 423</t>
           </r>
         </is>
       </c>
@@ -697,7 +697,7 @@
       <c r="C20" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">24 556</t>
+            <t xml:space="preserve">24 606</t>
           </r>
         </is>
       </c>
@@ -723,7 +723,7 @@
       <c r="C21" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">1 055 596</t>
+            <t xml:space="preserve">1 056 708</t>
           </r>
         </is>
       </c>
@@ -731,7 +731,7 @@
       <c r="E21" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">16.78</t>
+            <t xml:space="preserve">16.80</t>
           </r>
         </is>
       </c>
@@ -749,7 +749,7 @@
       <c r="C22" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">33 048</t>
+            <t xml:space="preserve">33 132</t>
           </r>
         </is>
       </c>
@@ -775,7 +775,7 @@
       <c r="C23" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">208 547</t>
+            <t xml:space="preserve">208 610</t>
           </r>
         </is>
       </c>
@@ -801,7 +801,7 @@
       <c r="C24" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">747 770</t>
+            <t xml:space="preserve">748 717</t>
           </r>
         </is>
       </c>
@@ -809,7 +809,7 @@
       <c r="E24" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">11.89</t>
+            <t xml:space="preserve">11.90</t>
           </r>
         </is>
       </c>
@@ -827,7 +827,7 @@
       <c r="C25" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">66 231</t>
+            <t xml:space="preserve">66 249</t>
           </r>
         </is>
       </c>
@@ -845,7 +845,7 @@
       <c r="A26" s="5" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">Dane do weryfikacji</t>
+            <t xml:space="preserve">DANE DO WERYFIKACJI</t>
           </r>
         </is>
       </c>
@@ -853,7 +853,7 @@
       <c r="C26" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">85 176</t>
+            <t xml:space="preserve">85 480</t>
           </r>
         </is>
       </c>
@@ -861,7 +861,7 @@
       <c r="E26" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">1.35</t>
+            <t xml:space="preserve">1.36</t>
           </r>
         </is>
       </c>
@@ -871,7 +871,7 @@
       <c r="A27" s="5" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">DANE DO WERYFIKACJI</t>
+            <t xml:space="preserve">Dane do weryfikacji</t>
           </r>
         </is>
       </c>
@@ -879,7 +879,7 @@
       <c r="C27" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">85 176</t>
+            <t xml:space="preserve">85 480</t>
           </r>
         </is>
       </c>
@@ -887,7 +887,7 @@
       <c r="E27" s="6" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">1.35</t>
+            <t xml:space="preserve">1.36</t>
           </r>
         </is>
       </c>
@@ -905,7 +905,7 @@
       <c r="C28" s="7" t="inlineStr"/>
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="8">
-        <v>46134.32026293967</v>
+        <v>46147.32025572937</v>
       </c>
       <c r="F28" s="8" t="inlineStr"/>
     </row>

</xml_diff>